<commit_message>
Modification URL et descriptions cac8c8b1878ba0624758cc6ec7846485b6701cdf
</commit_message>
<xml_diff>
--- a/ig/travaux-tru/StructureDefinition-esms-document-reference.xlsx
+++ b/ig/travaux-tru/StructureDefinition-esms-document-reference.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://esante.gouv.fr/fhir/ms/StructureDefinition/esms-document-reference</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/sdo-esms/esms-document-reference</t>
   </si>
   <si>
     <t>Version</t>
@@ -72,7 +72,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Suivi des orientations - pendant ESMS</t>
+    <t>Profil pour définir le dossier ESMS</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -102,7 +102,7 @@
     <t>Base Definition</t>
   </si>
   <si>
-    <t>http://esante.gouv.fr/fhir/ms/StructureDefinition/sdo-document-reference</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/sdo-esms/sdo-document-reference</t>
   </si>
   <si>
     <t>Abstract</t>

</xml_diff>